<commit_message>
Updated the first report.
</commit_message>
<xml_diff>
--- a/docs/Planilha de Horas.xlsx
+++ b/docs/Planilha de Horas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
   <si>
     <t>Total de Horas Gastas</t>
   </si>
@@ -65,6 +65,12 @@
   </si>
   <si>
     <t>Fazer os diagramas de entidadades</t>
+  </si>
+  <si>
+    <t>Criar o Front-End e o Back-End</t>
+  </si>
+  <si>
+    <t>Eleborar o primeiro relatório</t>
   </si>
 </sst>
 </file>
@@ -245,7 +251,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:F12" displayName="Project_tasks" name="Project_tasks" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:F14" displayName="Project_tasks" name="Project_tasks" id="1">
   <tableColumns count="6">
     <tableColumn name="Task" id="1"/>
     <tableColumn name="Priority" id="2"/>
@@ -475,7 +481,7 @@
       </c>
       <c r="C1" s="2">
         <f>SUM(Project_tasks[Spent Time])</f>
-        <v>0.3993055556</v>
+        <v>0.4409722222</v>
       </c>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
@@ -638,20 +644,44 @@
         <v>0.18055555555555555</v>
       </c>
     </row>
+    <row r="13" ht="22.5" customHeight="1">
+      <c r="A13" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="11">
+        <v>0.006944444444444444</v>
+      </c>
+    </row>
+    <row r="14" ht="22.5" customHeight="1">
+      <c r="A14" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="11">
+        <v>0.034722222222222224</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C1:D3"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="B7:B12">
+    <dataValidation type="list" allowBlank="1" sqref="B7:B14">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D7:D12">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D7:D14">
       <formula1>OR(NOT(ISERROR(DATEVALUE(D7))), AND(ISNUMBER(D7), LEFT(CELL("format", D7))="D"))</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="A7:A12 E7:E12"/>
-    <dataValidation type="list" allowBlank="1" sqref="C7:C12">
+    <dataValidation allowBlank="1" showDropDown="1" sqref="A7:A14 E7:E14"/>
+    <dataValidation type="list" allowBlank="1" sqref="C7:C14">
       <formula1>"Not started,In progress,Blocked,Completed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Updated the spreadsheet to track hours.
</commit_message>
<xml_diff>
--- a/docs/Planilha de Horas.xlsx
+++ b/docs/Planilha de Horas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="20">
   <si>
     <t>Total de Horas Gastas</t>
   </si>
@@ -55,22 +55,22 @@
     <t>Fazer os diagramas de estado</t>
   </si>
   <si>
-    <t>Not started</t>
-  </si>
-  <si>
     <t>Fazer os diagramas de Atividade</t>
   </si>
   <si>
+    <t>Fazer os diagramas de entidadades</t>
+  </si>
+  <si>
+    <t>Criar o Front-End e o Back-End</t>
+  </si>
+  <si>
+    <t>Eleborar o primeiro relatório</t>
+  </si>
+  <si>
+    <t>Atualizar o ERD com o estado dos simulados</t>
+  </si>
+  <si>
     <t>In progress</t>
-  </si>
-  <si>
-    <t>Fazer os diagramas de entidadades</t>
-  </si>
-  <si>
-    <t>Criar o Front-End e o Back-End</t>
-  </si>
-  <si>
-    <t>Eleborar o primeiro relatório</t>
   </si>
 </sst>
 </file>
@@ -251,7 +251,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:F14" displayName="Project_tasks" name="Project_tasks" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:F15" displayName="Project_tasks" name="Project_tasks" id="1">
   <tableColumns count="6">
     <tableColumn name="Task" id="1"/>
     <tableColumn name="Priority" id="2"/>
@@ -481,7 +481,7 @@
       </c>
       <c r="C1" s="2">
         <f>SUM(Project_tasks[Spent Time])</f>
-        <v>0.4409722222</v>
+        <v>0.4479166667</v>
       </c>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
@@ -600,7 +600,7 @@
         <v>8</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="10"/>
@@ -610,13 +610,13 @@
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="D11" s="9">
         <v>46066.0</v>
@@ -628,13 +628,13 @@
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>8</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="D12" s="9">
         <v>46062.0</v>
@@ -646,10 +646,14 @@
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
+        <v>16</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>9</v>
+      </c>
       <c r="D13" s="9"/>
       <c r="E13" s="10"/>
       <c r="F13" s="11">
@@ -658,14 +662,36 @@
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
+        <v>17</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>9</v>
+      </c>
       <c r="D14" s="9"/>
       <c r="E14" s="10"/>
       <c r="F14" s="11">
         <v>0.034722222222222224</v>
+      </c>
+    </row>
+    <row r="15" ht="22.5" customHeight="1">
+      <c r="A15" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="9">
+        <v>46087.0</v>
+      </c>
+      <c r="E15" s="10"/>
+      <c r="F15" s="11">
+        <v>0.006944444444444444</v>
       </c>
     </row>
   </sheetData>
@@ -674,14 +700,14 @@
     <mergeCell ref="C1:D3"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="B7:B14">
+    <dataValidation type="list" allowBlank="1" sqref="B7:B15">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D7:D14">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D7:D15">
       <formula1>OR(NOT(ISERROR(DATEVALUE(D7))), AND(ISNUMBER(D7), LEFT(CELL("format", D7))="D"))</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="A7:A14 E7:E14"/>
-    <dataValidation type="list" allowBlank="1" sqref="C7:C14">
+    <dataValidation allowBlank="1" showDropDown="1" sqref="A7:A15 E7:E15"/>
+    <dataValidation type="list" allowBlank="1" sqref="C7:C15">
       <formula1>"Not started,In progress,Blocked,Completed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Uploaded the Postgres DDL script and updated the spreadsheet to track hours.
</commit_message>
<xml_diff>
--- a/docs/Planilha de Horas.xlsx
+++ b/docs/Planilha de Horas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="26">
   <si>
     <t>Total de Horas Gastas</t>
   </si>
@@ -83,6 +83,12 @@
   </si>
   <si>
     <t>P1</t>
+  </si>
+  <si>
+    <t>Atualizar os schemas do script DDL e começar a criar as sessions</t>
+  </si>
+  <si>
+    <t>In progress</t>
   </si>
 </sst>
 </file>
@@ -266,7 +272,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:F18" displayName="Project_tasks" name="Project_tasks" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:F19" displayName="Project_tasks" name="Project_tasks" id="1">
   <tableColumns count="6">
     <tableColumn name="Task" id="1"/>
     <tableColumn name="Priority" id="2"/>
@@ -496,7 +502,7 @@
       </c>
       <c r="C1" s="2">
         <f>SUM(Project_tasks[Spent Time])</f>
-        <v>0.5833333333</v>
+        <v>0.6041666667</v>
       </c>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
@@ -759,20 +765,36 @@
         <v>0.003472222222222222</v>
       </c>
     </row>
+    <row r="19" ht="22.5" customHeight="1">
+      <c r="A19" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19" s="9"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="11">
+        <v>0.020833333333333332</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C1:D3"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="B7:B18">
+    <dataValidation type="list" allowBlank="1" sqref="B7:B19">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D7:D18">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D7:D19">
       <formula1>OR(NOT(ISERROR(DATEVALUE(D7))), AND(ISNUMBER(D7), LEFT(CELL("format", D7))="D"))</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="A7:A18 E7:E18"/>
-    <dataValidation type="list" allowBlank="1" sqref="C7:C18">
+    <dataValidation allowBlank="1" showDropDown="1" sqref="A7:A19 E7:E19"/>
+    <dataValidation type="list" allowBlank="1" sqref="C7:C19">
       <formula1>"Not started,In progress,Blocked,Completed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Updated the hours tracking spreadsheet.
</commit_message>
<xml_diff>
--- a/docs/Planilha de Horas.xlsx
+++ b/docs/Planilha de Horas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="25">
   <si>
     <t>Total de Horas Gastas</t>
   </si>
@@ -74,9 +74,6 @@
   </si>
   <si>
     <t>Criar os triggers e funções no Postgres</t>
-  </si>
-  <si>
-    <t>Not started</t>
   </si>
   <si>
     <t>Atualizar o ERD para ficar sincronizado com o script DDL</t>
@@ -502,7 +499,7 @@
       </c>
       <c r="C1" s="2">
         <f>SUM(Project_tasks[Spent Time])</f>
-        <v>0.6041666667</v>
+        <v>0.6666666667</v>
       </c>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
@@ -741,20 +738,22 @@
         <v>8</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="D17" s="9">
         <v>46088.0</v>
       </c>
       <c r="E17" s="10"/>
-      <c r="F17" s="11"/>
+      <c r="F17" s="11">
+        <v>0.0625</v>
+      </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>22</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>23</v>
       </c>
       <c r="C18" s="8" t="s">
         <v>9</v>
@@ -767,13 +766,13 @@
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="8" t="s">
         <v>24</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>25</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="10"/>

</xml_diff>

<commit_message>
Uploaded the 2nd report.
</commit_message>
<xml_diff>
--- a/docs/Planilha de Horas.xlsx
+++ b/docs/Planilha de Horas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="26">
   <si>
     <t>Total de Horas Gastas</t>
   </si>
@@ -82,10 +82,13 @@
     <t>P1</t>
   </si>
   <si>
-    <t>Atualizar os schemas do script DDL e começar a criar as sessions</t>
-  </si>
-  <si>
-    <t>In progress</t>
+    <t>Atualizar as tabelas do script DDL</t>
+  </si>
+  <si>
+    <t>Criar USERS e ROLES</t>
+  </si>
+  <si>
+    <t>Fazer o 2° relatório</t>
   </si>
 </sst>
 </file>
@@ -269,7 +272,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:F19" displayName="Project_tasks" name="Project_tasks" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:F21" displayName="Project_tasks" name="Project_tasks" id="1">
   <tableColumns count="6">
     <tableColumn name="Task" id="1"/>
     <tableColumn name="Priority" id="2"/>
@@ -499,7 +502,7 @@
       </c>
       <c r="C1" s="2">
         <f>SUM(Project_tasks[Spent Time])</f>
-        <v>0.6666666667</v>
+        <v>0.7777777778</v>
       </c>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
@@ -761,7 +764,7 @@
       <c r="D18" s="9"/>
       <c r="E18" s="10"/>
       <c r="F18" s="11">
-        <v>0.003472222222222222</v>
+        <v>0.010416666666666666</v>
       </c>
     </row>
     <row r="19" ht="22.5" customHeight="1">
@@ -772,12 +775,44 @@
         <v>22</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="10"/>
       <c r="F19" s="11">
         <v>0.020833333333333332</v>
+      </c>
+    </row>
+    <row r="20" ht="22.5" customHeight="1">
+      <c r="A20" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="9"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="11">
+        <v>0.0625</v>
+      </c>
+    </row>
+    <row r="21" ht="22.5" customHeight="1">
+      <c r="A21" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" s="9"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="11">
+        <v>0.041666666666666664</v>
       </c>
     </row>
   </sheetData>
@@ -786,14 +821,14 @@
     <mergeCell ref="C1:D3"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="B7:B19">
+    <dataValidation type="list" allowBlank="1" sqref="B7:B21">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D7:D19">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D7:D21">
       <formula1>OR(NOT(ISERROR(DATEVALUE(D7))), AND(ISNUMBER(D7), LEFT(CELL("format", D7))="D"))</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="A7:A19 E7:E19"/>
-    <dataValidation type="list" allowBlank="1" sqref="C7:C19">
+    <dataValidation allowBlank="1" showDropDown="1" sqref="A7:A21 E7:E21"/>
+    <dataValidation type="list" allowBlank="1" sqref="C7:C21">
       <formula1>"Not started,In progress,Blocked,Completed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs: update project tracking and database infrastructure scripts
- Add check-in-03 progress report and update hours spreadsheet.
- Include custom PostgreSQL casts for handling C# Enums.
- Update database creation and privileges scripts to reflect RBAC changes.
</commit_message>
<xml_diff>
--- a/docs/Planilha de Horas.xlsx
+++ b/docs/Planilha de Horas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="40">
   <si>
     <t>Total de Horas Gastas</t>
   </si>
@@ -89,6 +89,62 @@
   </si>
   <si>
     <t>Fazer o 2° relatório</t>
+  </si>
+  <si>
+    <t>Implementação de Persistência de Sessão Distribuída</t>
+  </si>
+  <si>
+    <t>Desenvolvimento da lógica de persistência de sessão utilizando PostgreSQL como cache distribuído e integração com o middleware do ASP.NET Core.</t>
+  </si>
+  <si>
+    <t>Normalização de Tipos Primitivos e Mapping de Enums no EF Core</t>
+  </si>
+  <si>
+    <t>Configuração de mapeamento de tipos enums nativos do PostgreSQL para tipos C# e implementação de Casting de dados.</t>
+  </si>
+  <si>
+    <t>Desenvolvimento de um sistema de autorização baseado em políticas de acesso.</t>
+  </si>
+  <si>
+    <t>Criação de AuthorizationHandlers e PolicyProviders para controle de acesso no backend.</t>
+  </si>
+  <si>
+    <t>Refatoração do projeto para Domain-Driven Design (DDD)</t>
+  </si>
+  <si>
+    <t>Separação de entidades de domínio da camada de persistência.</t>
+  </si>
+  <si>
+    <t>Modelagem e Implementação de RBAC (Role-Based Access Control)</t>
+  </si>
+  <si>
+    <t>Mapeamento de relacionamentos Muitos-para-Muitos entre Usuários, Roles e Permissões no banco de dados.</t>
+  </si>
+  <si>
+    <t>Planejamento de Testes de Unitários</t>
+  </si>
+  <si>
+    <t>In progress</t>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t xml:space="preserve">Desenvolvimento de Testes Unitários com TestContainers com PostgreSQL e </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>ASP.NET</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> Core</t>
+    </r>
+  </si>
+  <si>
+    <t>Desenvolimento do 2° Relatório</t>
   </si>
 </sst>
 </file>
@@ -98,7 +154,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd&quot;/&quot;mm&quot;/&quot;yyyy"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -125,6 +181,11 @@
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+      <name val="Roboto"/>
     </font>
   </fonts>
   <fills count="4">
@@ -153,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -192,6 +253,12 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -272,7 +339,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:F21" displayName="Project_tasks" name="Project_tasks" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:F28" displayName="Project_tasks" name="Project_tasks" id="1">
   <tableColumns count="6">
     <tableColumn name="Task" id="1"/>
     <tableColumn name="Priority" id="2"/>
@@ -502,7 +569,7 @@
       </c>
       <c r="C1" s="2">
         <f>SUM(Project_tasks[Spent Time])</f>
-        <v>0.7777777778</v>
+        <v>1.565972222</v>
       </c>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
@@ -815,26 +882,153 @@
         <v>0.041666666666666664</v>
       </c>
     </row>
+    <row r="22" ht="22.5" customHeight="1">
+      <c r="A22" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="9"/>
+      <c r="E22" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F22" s="11">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="23" ht="22.5" customHeight="1">
+      <c r="A23" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="9"/>
+      <c r="E23" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F23" s="11">
+        <v>0.034722222222222224</v>
+      </c>
+    </row>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="A24" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" s="9"/>
+      <c r="E24" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F24" s="11">
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25" s="9"/>
+      <c r="E25" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F25" s="11">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="26" ht="22.5" customHeight="1">
+      <c r="A26" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="9"/>
+      <c r="E26" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F26" s="11">
+        <v>0.04513888888888889</v>
+      </c>
+    </row>
+    <row r="27" ht="22.5" customHeight="1">
+      <c r="A27" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D27" s="9"/>
+      <c r="E27" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="F27" s="11">
+        <v>0.006944444444444444</v>
+      </c>
+    </row>
+    <row r="28" ht="22.5" customHeight="1">
+      <c r="A28" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" s="9"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="11">
+        <v>0.034722222222222224</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C1:D3"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="B7:B21">
+    <dataValidation type="list" allowBlank="1" sqref="B7:B28">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D7:D21">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D7:D28">
       <formula1>OR(NOT(ISERROR(DATEVALUE(D7))), AND(ISNUMBER(D7), LEFT(CELL("format", D7))="D"))</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="A7:A21 E7:E21"/>
-    <dataValidation type="list" allowBlank="1" sqref="C7:C21">
+    <dataValidation allowBlank="1" showDropDown="1" sqref="A7:A28 E7:E28"/>
+    <dataValidation type="list" allowBlank="1" sqref="C7:C28">
       <formula1>"Not started,In progress,Blocked,Completed"</formula1>
     </dataValidation>
   </dataValidations>
-  <drawing r:id="rId1"/>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="E27"/>
+  </hyperlinks>
+  <drawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update hours spreadsheet and upload report 4.
</commit_message>
<xml_diff>
--- a/docs/Planilha de Horas.xlsx
+++ b/docs/Planilha de Horas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="58">
   <si>
     <t>Total de Horas Gastas</t>
   </si>
@@ -121,15 +121,12 @@
     <t>Mapeamento de relacionamentos Muitos-para-Muitos entre Usuários, Roles e Permissões no banco de dados.</t>
   </si>
   <si>
-    <t>Planejamento de Testes de Unitários</t>
-  </si>
-  <si>
-    <t>In progress</t>
+    <t>Planejamento de Testes de Integração</t>
   </si>
   <si>
     <r>
       <rPr/>
-      <t xml:space="preserve">Desenvolvimento de Testes Unitários com TestContainers com PostgreSQL e </t>
+      <t xml:space="preserve">Desenvolvimento de Testes de Integração com TestContainers com PostgreSQL e </t>
     </r>
     <r>
       <rPr>
@@ -145,6 +142,63 @@
   </si>
   <si>
     <t>Desenvolimento do 2° Relatório</t>
+  </si>
+  <si>
+    <t>Sistema de Convite</t>
+  </si>
+  <si>
+    <t>Implementação de fluxo administrativo que permite a geração de códigos únicos para convite de novos usuários com cargos específicos.</t>
+  </si>
+  <si>
+    <t>Implementaçãod de TestContainers</t>
+  </si>
+  <si>
+    <t>Configuração e debugging do ambiente Docker para instanciar bancos PostgreSQL efêmeros durante a execução dos testes.</t>
+  </si>
+  <si>
+    <t>Ciclo de Vida (IAsyncLifetime)</t>
+  </si>
+  <si>
+    <t>Implementação de setup e teardown assíncronos para garantir o isolamento atômico de cada caso de teste.</t>
+  </si>
+  <si>
+    <t>Limpeza de Dados (Respawn)</t>
+  </si>
+  <si>
+    <t>Integração da biblioteca Respawn para resetar o estado do banco entre os testes sem necessidade de recriar o container.</t>
+  </si>
+  <si>
+    <t>Refatoração do AuthController</t>
+  </si>
+  <si>
+    <t>Ajuste do controlador de autenticação para suportar os requisitos dos testes de integração e correção de fluxos de login/registro.</t>
+  </si>
+  <si>
+    <t>Segurança e Autorização Customizada</t>
+  </si>
+  <si>
+    <t>Implementação de um Authentication Scheme customizado com um Session Authorization Handler. Esta mudança foi crucial para resolver erros de 405 Method Not Allowed e substituir a autenticação padrão baseada em cookies por uma lógica vinculada à sessão do sistema.</t>
+  </si>
+  <si>
+    <t>Serviço de Questões (Question Service)</t>
+  </si>
+  <si>
+    <t>Implementação de busca com Paged Response (respostas paginadas). Uso extensivo de IQueryable e QueryableExtensions para filtragem eficiente. Criação de um objeto de filtro de consulta (Question Query Filter) para buscas dinâmicas.</t>
+  </si>
+  <si>
+    <t>Mapeamento de Enums no PostgreSQL</t>
+  </si>
+  <si>
+    <t>Refatoração da configuração do NpgsqlDataSource no .NET 9 para suporte nativo a tipos enumerados no banco de dados.</t>
+  </si>
+  <si>
+    <t>População de Dados</t>
+  </si>
+  <si>
+    <t>Script Python utilizando psycopg2 para ingestão de questões via API externa para a base de dados local.</t>
+  </si>
+  <si>
+    <t>Relatório 4</t>
   </si>
 </sst>
 </file>
@@ -339,7 +393,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:F28" displayName="Project_tasks" name="Project_tasks" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:F38" displayName="Project_tasks" name="Project_tasks" id="1">
   <tableColumns count="6">
     <tableColumn name="Task" id="1"/>
     <tableColumn name="Priority" id="2"/>
@@ -569,7 +623,7 @@
       </c>
       <c r="C1" s="2">
         <f>SUM(Project_tasks[Spent Time])</f>
-        <v>1.565972222</v>
+        <v>2.458333333</v>
       </c>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
@@ -980,11 +1034,11 @@
         <v>22</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="D27" s="9"/>
       <c r="E27" s="13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F27" s="11">
         <v>0.006944444444444444</v>
@@ -992,7 +1046,7 @@
     </row>
     <row r="28" ht="22.5" customHeight="1">
       <c r="A28" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B28" s="8" t="s">
         <v>22</v>
@@ -1004,6 +1058,184 @@
       <c r="E28" s="14"/>
       <c r="F28" s="11">
         <v>0.034722222222222224</v>
+      </c>
+    </row>
+    <row r="29" ht="22.5" customHeight="1">
+      <c r="A29" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="9"/>
+      <c r="E29" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="F29" s="11">
+        <v>0.09722222222222222</v>
+      </c>
+    </row>
+    <row r="30" ht="22.5" customHeight="1">
+      <c r="A30" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="9"/>
+      <c r="E30" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="F30" s="11">
+        <v>0.12152777777777778</v>
+      </c>
+    </row>
+    <row r="31" ht="22.5" customHeight="1">
+      <c r="A31" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" s="9"/>
+      <c r="E31" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="F31" s="11">
+        <v>0.03125</v>
+      </c>
+    </row>
+    <row r="32" ht="22.5" customHeight="1">
+      <c r="A32" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32" s="9"/>
+      <c r="E32" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="F32" s="11">
+        <v>0.16666666666666666</v>
+      </c>
+    </row>
+    <row r="33" ht="22.5" customHeight="1">
+      <c r="A33" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33" s="9"/>
+      <c r="E33" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="F33" s="11">
+        <v>0.10416666666666667</v>
+      </c>
+    </row>
+    <row r="34" ht="22.5" customHeight="1">
+      <c r="A34" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="F34" s="11">
+        <v>0.041666666666666664</v>
+      </c>
+    </row>
+    <row r="35" ht="22.5" customHeight="1">
+      <c r="A35" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D35" s="9"/>
+      <c r="E35" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="F35" s="11">
+        <v>0.1909722222222222</v>
+      </c>
+    </row>
+    <row r="36" ht="22.5" customHeight="1">
+      <c r="A36" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D36" s="9"/>
+      <c r="E36" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="F36" s="11">
+        <v>0.013888888888888888</v>
+      </c>
+    </row>
+    <row r="37" ht="22.5" customHeight="1">
+      <c r="A37" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D37" s="9"/>
+      <c r="E37" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="F37" s="11">
+        <v>0.10069444444444445</v>
+      </c>
+    </row>
+    <row r="38" ht="22.5" customHeight="1">
+      <c r="A38" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D38" s="9"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="11">
+        <v>0.024305555555555556</v>
       </c>
     </row>
   </sheetData>
@@ -1012,14 +1244,14 @@
     <mergeCell ref="C1:D3"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="B7:B28">
+    <dataValidation type="list" allowBlank="1" sqref="B7:B38">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D7:D28">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D7:D38">
       <formula1>OR(NOT(ISERROR(DATEVALUE(D7))), AND(ISNUMBER(D7), LEFT(CELL("format", D7))="D"))</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="A7:A28 E7:E28"/>
-    <dataValidation type="list" allowBlank="1" sqref="C7:C28">
+    <dataValidation allowBlank="1" showDropDown="1" sqref="A7:A38 E7:E38"/>
+    <dataValidation type="list" allowBlank="1" sqref="C7:C38">
       <formula1>"Not started,In progress,Blocked,Completed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add last report before final deadline.
</commit_message>
<xml_diff>
--- a/docs/Planilha de Horas.xlsx
+++ b/docs/Planilha de Horas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="93">
   <si>
     <t>Total de Horas Gastas</t>
   </si>
@@ -199,6 +199,111 @@
   </si>
   <si>
     <t>Relatório 4</t>
+  </si>
+  <si>
+    <t>Global Exception Handling Middleware</t>
+  </si>
+  <si>
+    <t>Implementação de um Middleware para cuidar de Excessões inesperadas da infraestrutura de forma segura.</t>
+  </si>
+  <si>
+    <t>Result Pattern</t>
+  </si>
+  <si>
+    <t>Implementação da arquitetura genérica `Result&lt;T&gt;`, método extensão `Match` para ser usado nos controlers e refatoração dos blocos de código principais para remover `exception-throwing` para regras de negócio.</t>
+  </si>
+  <si>
+    <t>Saved Question Service, Controller e Paginatação</t>
+  </si>
+  <si>
+    <t>Implementação das rotas do Controller, implementação do serviço com o backend com o `IQueryable` que serve dados eficientemente para o frontend.</t>
+  </si>
+  <si>
+    <t>Saved Questions Database Mapping &amp; EF Migration</t>
+  </si>
+  <si>
+    <t>Definição das relações em `SavedQuestionConfiguration`, adcionado um `DbSet` ao `DbContext`, execução e aplicação da migração EF.</t>
+  </si>
+  <si>
+    <t>User Goal Controller e Serviços</t>
+  </si>
+  <si>
+    <t>Design as regras de domínio para as métricas do estudante, processando a regra de négocio (como enforçar o limite de um objetivo), e a criação das rotas correspondentes.</t>
+  </si>
+  <si>
+    <t>Subjects Service, Controller</t>
+  </si>
+  <si>
+    <t>Foi contruído o serviço `SubjectService` e controller `SubjectsController`.</t>
+  </si>
+  <si>
+    <t>Refatoração do SolvedQuestionDto</t>
+  </si>
+  <si>
+    <t>Adicionar enunciado, alternativa correta e escolhida ao SolvedQuestionDto.</t>
+  </si>
+  <si>
+    <t>Refatoração do SolvedQuestionsService</t>
+  </si>
+  <si>
+    <t>Vários controllers estavam usando as funcionalidades de converter STRING para JsonElement, então a solução encontrada foi criar métodos de extensão para algumas classes como `Question` model.</t>
+  </si>
+  <si>
+    <t>Implementação do SavedQuestionService</t>
+  </si>
+  <si>
+    <t>Foi implementado um serviço que permite ao usuário salvar questões para revisar mais tarde.</t>
+  </si>
+  <si>
+    <t>SavedQuestionsController</t>
+  </si>
+  <si>
+    <t>Implementação das rotas do `SavedQuestionService`.</t>
+  </si>
+  <si>
+    <t>Planejamento dos próximos passos</t>
+  </si>
+  <si>
+    <t>Planejamento da entrega final com os items prioritários e essenciais.</t>
+  </si>
+  <si>
+    <t>Exams Service</t>
+  </si>
+  <si>
+    <t>Implementação de um serviço complexo de simulados, que têm persistência de respostas e avaliação do desempenho do estudante de forma mais realista possível.</t>
+  </si>
+  <si>
+    <t>Exams Controller</t>
+  </si>
+  <si>
+    <t>Implementação das rotas do serviço `ExamsService`.</t>
+  </si>
+  <si>
+    <t>UserPreferences Service &amp; Controller</t>
+  </si>
+  <si>
+    <t>Implementação de um serviço e controller para as preferências do usuário.</t>
+  </si>
+  <si>
+    <t>Scaffold e configuarção do Front-End</t>
+  </si>
+  <si>
+    <t>Scaffold com Next, shadcn/ui e tailwind, começo da implementação da sidebar.</t>
+  </si>
+  <si>
+    <t>Funcionalidade UserService</t>
+  </si>
+  <si>
+    <t>Foi implementado um método ao serviço do usuário que permite buscar informações sobre um usuário específico e a implementação da rota no controller.</t>
+  </si>
+  <si>
+    <t>Solução dos problemas com Enums</t>
+  </si>
+  <si>
+    <t>Através da implementação de Value Converters customizados no EF Core, garantindo compatibilidade com APIs externas em português.</t>
+  </si>
+  <si>
+    <t>Relatório 5</t>
   </si>
 </sst>
 </file>
@@ -393,7 +498,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:F38" displayName="Project_tasks" name="Project_tasks" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:F56" displayName="Project_tasks" name="Project_tasks" id="1">
   <tableColumns count="6">
     <tableColumn name="Task" id="1"/>
     <tableColumn name="Priority" id="2"/>
@@ -623,7 +728,7 @@
       </c>
       <c r="C1" s="2">
         <f>SUM(Project_tasks[Spent Time])</f>
-        <v>2.458333333</v>
+        <v>3.65625</v>
       </c>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
@@ -1238,20 +1343,342 @@
         <v>0.024305555555555556</v>
       </c>
     </row>
+    <row r="39" ht="22.5" customHeight="1">
+      <c r="A39" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D39" s="9"/>
+      <c r="E39" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="F39" s="11">
+        <v>0.041666666666666664</v>
+      </c>
+    </row>
+    <row r="40" ht="22.5" customHeight="1">
+      <c r="A40" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D40" s="9"/>
+      <c r="E40" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="F40" s="11">
+        <v>0.052083333333333336</v>
+      </c>
+    </row>
+    <row r="41" ht="22.5" customHeight="1">
+      <c r="A41" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D41" s="9"/>
+      <c r="E41" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="F41" s="11">
+        <v>0.09375</v>
+      </c>
+    </row>
+    <row r="42" ht="22.5" customHeight="1">
+      <c r="A42" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D42" s="9"/>
+      <c r="E42" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F42" s="11">
+        <v>0.020833333333333332</v>
+      </c>
+    </row>
+    <row r="43" ht="22.5" customHeight="1">
+      <c r="A43" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D43" s="9"/>
+      <c r="E43" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="F43" s="11">
+        <v>0.0625</v>
+      </c>
+    </row>
+    <row r="44" ht="22.5" customHeight="1">
+      <c r="A44" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D44" s="9"/>
+      <c r="E44" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="F44" s="11">
+        <v>0.0625</v>
+      </c>
+    </row>
+    <row r="45" ht="22.5" customHeight="1">
+      <c r="A45" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D45" s="9"/>
+      <c r="E45" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="F45" s="11">
+        <v>0.052083333333333336</v>
+      </c>
+    </row>
+    <row r="46" ht="22.5" customHeight="1">
+      <c r="A46" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D46" s="9"/>
+      <c r="E46" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="F46" s="11">
+        <v>0.010416666666666666</v>
+      </c>
+    </row>
+    <row r="47" ht="22.5" customHeight="1">
+      <c r="A47" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D47" s="9"/>
+      <c r="E47" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="F47" s="11">
+        <v>0.03125</v>
+      </c>
+    </row>
+    <row r="48" ht="22.5" customHeight="1">
+      <c r="A48" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D48" s="9"/>
+      <c r="E48" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="F48" s="11">
+        <v>0.027777777777777776</v>
+      </c>
+    </row>
+    <row r="49" ht="22.5" customHeight="1">
+      <c r="A49" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D49" s="9"/>
+      <c r="E49" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="F49" s="11">
+        <v>0.052083333333333336</v>
+      </c>
+    </row>
+    <row r="50" ht="22.5" customHeight="1">
+      <c r="A50" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D50" s="9"/>
+      <c r="E50" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="F50" s="11">
+        <v>0.3194444444444444</v>
+      </c>
+    </row>
+    <row r="51" ht="22.5" customHeight="1">
+      <c r="A51" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D51" s="9"/>
+      <c r="E51" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="F51" s="11">
+        <v>0.034722222222222224</v>
+      </c>
+    </row>
+    <row r="52" ht="22.5" customHeight="1">
+      <c r="A52" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D52" s="9"/>
+      <c r="E52" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="F52" s="11">
+        <v>0.027777777777777776</v>
+      </c>
+    </row>
+    <row r="53" ht="22.5" customHeight="1">
+      <c r="A53" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="B53" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D53" s="9"/>
+      <c r="E53" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="F53" s="11">
+        <v>0.19444444444444445</v>
+      </c>
+    </row>
+    <row r="54" ht="22.5" customHeight="1">
+      <c r="A54" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D54" s="9"/>
+      <c r="E54" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="F54" s="11">
+        <v>0.020833333333333332</v>
+      </c>
+    </row>
+    <row r="55" ht="22.5" customHeight="1">
+      <c r="A55" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="B55" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D55" s="9"/>
+      <c r="E55" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="F55" s="11">
+        <v>0.04513888888888889</v>
+      </c>
+    </row>
+    <row r="56" ht="22.5" customHeight="1">
+      <c r="A56" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D56" s="9"/>
+      <c r="E56" s="14"/>
+      <c r="F56" s="11">
+        <v>0.04861111111111111</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:B3"/>
     <mergeCell ref="C1:D3"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="B7:B38">
+    <dataValidation type="list" allowBlank="1" sqref="B7:B56">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D7:D38">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D7:D56">
       <formula1>OR(NOT(ISERROR(DATEVALUE(D7))), AND(ISNUMBER(D7), LEFT(CELL("format", D7))="D"))</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="A7:A38 E7:E38"/>
-    <dataValidation type="list" allowBlank="1" sqref="C7:C38">
+    <dataValidation allowBlank="1" showDropDown="1" sqref="A7:A56 E7:E56"/>
+    <dataValidation type="list" allowBlank="1" sqref="C7:C56">
       <formula1>"Not started,In progress,Blocked,Completed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>